<commit_message>
Excel line: built and tested in Excel for Microsoft 365
</commit_message>
<xml_diff>
--- a/Work Tracker Demo.xlsx
+++ b/Work Tracker Demo.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B8C046DA-E49E-4C7E-B805-181713F9980E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DBCB23F0-C766-4B66-9BCA-B2DA2543DB32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9621E1EE-779C-450F-87AC-5CDFDDD3B01E}"/>
+    <workbookView xWindow="0" yWindow="1305" windowWidth="21600" windowHeight="11520" xr2:uid="{1F9FEBDE-B559-42F3-97A0-796F3DC4A106}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -548,13 +548,13 @@
     <t>Good to know</t>
   </si>
   <si>
-    <t>Nothing here needs macros. The file works in Excel 2010 and later, including Microsoft 365.</t>
+    <t>Nothing here needs macros. It uses formulas that exist in Excel 2010 and later; built and tested in Excel for Microsoft 365 on Windows.</t>
   </si>
   <si>
     <t>The Lists sheet holds helper formulas for the dashboard. Leave it as it is.</t>
   </si>
   <si>
-    <t>The sample dates were set on Oct 2, 2026, so some tasks were overdue and some due that week. The dashboard always compares with today's date, so the counts move as days pass.</t>
+    <t>The sample dates were set on Oct 6, 2026, so some tasks were overdue and some due that week. The dashboard always compares with today's date, so the counts move as days pass.</t>
   </si>
 </sst>
 </file>
@@ -1010,7 +1010,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
-    <tableStyle name="AZG Table" pivot="0" table="0" count="2" xr9:uid="{152807FA-F056-43F9-8DBA-FF331AEB0691}">
+    <tableStyle name="AZG Table" pivot="0" table="0" count="2" xr9:uid="{A2000176-35D8-4FC9-8680-BCB2C491144B}">
       <tableStyleElement type="wholeTable" dxfId="19"/>
       <tableStyleElement type="headerRow" dxfId="18"/>
     </tableStyle>
@@ -1027,22 +1027,22 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{49590DEB-0070-423E-982E-B237A19237B5}" name="Tasks" displayName="Tasks" ref="A1:K43" totalsRowShown="0" headerRowDxfId="14">
-  <autoFilter ref="A1:K43" xr:uid="{49590DEB-0070-423E-982E-B237A19237B5}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C309CA55-1D5B-4171-95B2-225A5B757F40}" name="Tasks" displayName="Tasks" ref="A1:K43" totalsRowShown="0" headerRowDxfId="14">
+  <autoFilter ref="A1:K43" xr:uid="{C309CA55-1D5B-4171-95B2-225A5B757F40}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{F7799466-306B-4085-88A3-9BAFC2E2963B}" name="ID" dataDxfId="15"/>
-    <tableColumn id="2" xr3:uid="{515B7545-E5A6-4900-BB7B-2FBE4FB6AAAF}" name="Task"/>
-    <tableColumn id="3" xr3:uid="{B35098B6-DA25-4832-AEA0-570CE5C79917}" name="Owner"/>
-    <tableColumn id="4" xr3:uid="{A2138601-112D-4AC2-B4EE-BE5361088E3A}" name="Department"/>
-    <tableColumn id="5" xr3:uid="{F0814445-79E8-4D6E-834F-EB0C3725F3D6}" name="Status"/>
-    <tableColumn id="6" xr3:uid="{2E7DEBD4-F428-4726-B2CF-4B4DE5C6E0BE}" name="Priority"/>
-    <tableColumn id="7" xr3:uid="{E80337C6-3463-456A-B55A-DCB248D25985}" name="Start" dataDxfId="17"/>
-    <tableColumn id="8" xr3:uid="{5E3602ED-F95C-4854-BA13-F13471ACD221}" name="Due" dataDxfId="16"/>
-    <tableColumn id="9" xr3:uid="{81E0FB5F-7848-475F-8608-DF0EBF9C3069}" name="% Complete" dataDxfId="13"/>
-    <tableColumn id="10" xr3:uid="{5E664E38-2C8D-4F49-88D8-0A7E555C94E1}" name="Year" dataDxfId="12">
+    <tableColumn id="1" xr3:uid="{95AE37A2-8FAF-401A-B1E7-3C4D9F4C769C}" name="ID" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{7C6E9FE7-90F0-4387-AA2D-FFB5CBE04370}" name="Task"/>
+    <tableColumn id="3" xr3:uid="{D26EEC67-5C02-42A3-9CD5-9586411A4B4F}" name="Owner"/>
+    <tableColumn id="4" xr3:uid="{6CC9D32B-6B50-4C3A-9D8F-EAF44DE4BC33}" name="Department"/>
+    <tableColumn id="5" xr3:uid="{57DD70EF-1F9B-44E5-A5F3-9A29FFD7F595}" name="Status"/>
+    <tableColumn id="6" xr3:uid="{9ED822FD-A86B-4DA2-BE22-0869F8E3A98E}" name="Priority"/>
+    <tableColumn id="7" xr3:uid="{0E7840EE-FBBE-42DE-BC77-A61A12EA26FA}" name="Start" dataDxfId="17"/>
+    <tableColumn id="8" xr3:uid="{60854EE4-9596-44B4-9B30-43C6545612F8}" name="Due" dataDxfId="16"/>
+    <tableColumn id="9" xr3:uid="{94837B56-72C6-47E5-88CD-4FE62E94847D}" name="% Complete" dataDxfId="13"/>
+    <tableColumn id="10" xr3:uid="{5EB4190D-2789-47DC-ADDE-D5641105789D}" name="Year" dataDxfId="12">
       <calculatedColumnFormula>IF(Tasks[[#This Row],[Due]]="","",YEAR(Tasks[[#This Row],[Due]]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{1DD86DAE-03BB-432E-82AB-37C133F30EC1}" name="Notes"/>
+    <tableColumn id="11" xr3:uid="{28387B19-2D1A-41E3-AE15-9A1E0CB32EB6}" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="AZG Table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1344,7 +1344,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11EDC162-3DBE-44AD-8899-AC75CDC4CA74}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46D28430-7EC2-42C2-B6D5-BD508157B9BC}">
   <sheetPr>
     <tabColor rgb="FF1F3A5F"/>
     <pageSetUpPr fitToPage="1"/>
@@ -1418,7 +1418,7 @@
       <c r="A3" s="6"/>
       <c r="B3" s="16" t="str">
         <f ca="1">"As of "&amp;TEXT(TODAY(),"ddd, mmm d, yyyy")&amp;"   |   Pick an owner, status or year: the whole page follows."</f>
-        <v>As of Fri, Oct 2, 2026   |   Pick an owner, status or year: the whole page follows.</v>
+        <v>As of Tue, Oct 6, 2026   |   Pick an owner, status or year: the whole page follows.</v>
       </c>
       <c r="C3" s="6"/>
       <c r="D3" s="6"/>
@@ -1696,7 +1696,7 @@
       <c r="A13" s="6"/>
       <c r="B13" s="33">
         <f>IF(Lists!$Q4="","",IF(MOD(INT(Lists!$P4),100000)=99999,"",MOD(INT(Lists!$P4),100000)))</f>
-        <v>46282</v>
+        <v>46286</v>
       </c>
       <c r="C13" s="6" t="str">
         <f>IF(Lists!$Q4="","No tasks match these filters",INDEX(Tasks[Task],Lists!$Q4)&amp;"")</f>
@@ -1733,7 +1733,7 @@
       <c r="K13" s="6"/>
       <c r="L13" s="33">
         <f ca="1">IF(Lists!$I4="","",INT(Lists!$H4))</f>
-        <v>46297</v>
+        <v>46301</v>
       </c>
       <c r="M13" s="6" t="str">
         <f ca="1">IF(Lists!$I4="","Nothing due in the next 7 days",INDEX(Tasks[Task],Lists!$I4)&amp;"")</f>
@@ -1761,7 +1761,7 @@
       <c r="A14" s="6"/>
       <c r="B14" s="33">
         <f>IF(Lists!$Q5="","",IF(MOD(INT(Lists!$P5),100000)=99999,"",MOD(INT(Lists!$P5),100000)))</f>
-        <v>46285</v>
+        <v>46289</v>
       </c>
       <c r="C14" s="6" t="str">
         <f>IF(Lists!$Q5="","",INDEX(Tasks[Task],Lists!$Q5)&amp;"")</f>
@@ -1798,7 +1798,7 @@
       <c r="K14" s="6"/>
       <c r="L14" s="33">
         <f ca="1">IF(Lists!$I5="","",INT(Lists!$H5))</f>
-        <v>46298</v>
+        <v>46302</v>
       </c>
       <c r="M14" s="6" t="str">
         <f ca="1">IF(Lists!$I5="","",INDEX(Tasks[Task],Lists!$I5)&amp;"")</f>
@@ -1826,7 +1826,7 @@
       <c r="A15" s="6"/>
       <c r="B15" s="33">
         <f>IF(Lists!$Q6="","",IF(MOD(INT(Lists!$P6),100000)=99999,"",MOD(INT(Lists!$P6),100000)))</f>
-        <v>46289</v>
+        <v>46293</v>
       </c>
       <c r="C15" s="6" t="str">
         <f>IF(Lists!$Q6="","",INDEX(Tasks[Task],Lists!$Q6)&amp;"")</f>
@@ -1863,7 +1863,7 @@
       <c r="K15" s="6"/>
       <c r="L15" s="33">
         <f ca="1">IF(Lists!$I6="","",INT(Lists!$H6))</f>
-        <v>46299</v>
+        <v>46303</v>
       </c>
       <c r="M15" s="6" t="str">
         <f ca="1">IF(Lists!$I6="","",INDEX(Tasks[Task],Lists!$I6)&amp;"")</f>
@@ -1891,7 +1891,7 @@
       <c r="A16" s="6"/>
       <c r="B16" s="33">
         <f>IF(Lists!$Q7="","",IF(MOD(INT(Lists!$P7),100000)=99999,"",MOD(INT(Lists!$P7),100000)))</f>
-        <v>46291</v>
+        <v>46295</v>
       </c>
       <c r="C16" s="6" t="str">
         <f>IF(Lists!$Q7="","",INDEX(Tasks[Task],Lists!$Q7)&amp;"")</f>
@@ -1928,7 +1928,7 @@
       <c r="K16" s="6"/>
       <c r="L16" s="33">
         <f ca="1">IF(Lists!$I7="","",INT(Lists!$H7))</f>
-        <v>46300</v>
+        <v>46304</v>
       </c>
       <c r="M16" s="6" t="str">
         <f ca="1">IF(Lists!$I7="","",INDEX(Tasks[Task],Lists!$I7)&amp;"")</f>
@@ -1956,7 +1956,7 @@
       <c r="A17" s="6"/>
       <c r="B17" s="33">
         <f>IF(Lists!$Q8="","",IF(MOD(INT(Lists!$P8),100000)=99999,"",MOD(INT(Lists!$P8),100000)))</f>
-        <v>46293</v>
+        <v>46297</v>
       </c>
       <c r="C17" s="6" t="str">
         <f>IF(Lists!$Q8="","",INDEX(Tasks[Task],Lists!$Q8)&amp;"")</f>
@@ -1993,7 +1993,7 @@
       <c r="K17" s="6"/>
       <c r="L17" s="33">
         <f ca="1">IF(Lists!$I8="","",INT(Lists!$H8))</f>
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="M17" s="6" t="str">
         <f ca="1">IF(Lists!$I8="","",INDEX(Tasks[Task],Lists!$I8)&amp;"")</f>
@@ -2021,7 +2021,7 @@
       <c r="A18" s="6"/>
       <c r="B18" s="33">
         <f>IF(Lists!$Q9="","",IF(MOD(INT(Lists!$P9),100000)=99999,"",MOD(INT(Lists!$P9),100000)))</f>
-        <v>46295</v>
+        <v>46299</v>
       </c>
       <c r="C18" s="6" t="str">
         <f>IF(Lists!$Q9="","",INDEX(Tasks[Task],Lists!$Q9)&amp;"")</f>
@@ -2058,7 +2058,7 @@
       <c r="K18" s="6"/>
       <c r="L18" s="33">
         <f ca="1">IF(Lists!$I9="","",INT(Lists!$H9))</f>
-        <v>46303</v>
+        <v>46307</v>
       </c>
       <c r="M18" s="6" t="str">
         <f ca="1">IF(Lists!$I9="","",INDEX(Tasks[Task],Lists!$I9)&amp;"")</f>
@@ -2086,7 +2086,7 @@
       <c r="A19" s="6"/>
       <c r="B19" s="33">
         <f>IF(Lists!$Q10="","",IF(MOD(INT(Lists!$P10),100000)=99999,"",MOD(INT(Lists!$P10),100000)))</f>
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="C19" s="6" t="str">
         <f>IF(Lists!$Q10="","",INDEX(Tasks[Task],Lists!$Q10)&amp;"")</f>
@@ -2151,7 +2151,7 @@
       <c r="A20" s="6"/>
       <c r="B20" s="33">
         <f>IF(Lists!$Q11="","",IF(MOD(INT(Lists!$P11),100000)=99999,"",MOD(INT(Lists!$P11),100000)))</f>
-        <v>46297</v>
+        <v>46301</v>
       </c>
       <c r="C20" s="6" t="str">
         <f>IF(Lists!$Q11="","",INDEX(Tasks[Task],Lists!$Q11)&amp;"")</f>
@@ -2216,7 +2216,7 @@
       <c r="A21" s="6"/>
       <c r="B21" s="33">
         <f>IF(Lists!$Q12="","",IF(MOD(INT(Lists!$P12),100000)=99999,"",MOD(INT(Lists!$P12),100000)))</f>
-        <v>46298</v>
+        <v>46302</v>
       </c>
       <c r="C21" s="6" t="str">
         <f>IF(Lists!$Q12="","",INDEX(Tasks[Task],Lists!$Q12)&amp;"")</f>
@@ -2266,7 +2266,7 @@
       <c r="A22" s="6"/>
       <c r="B22" s="33">
         <f>IF(Lists!$Q13="","",IF(MOD(INT(Lists!$P13),100000)=99999,"",MOD(INT(Lists!$P13),100000)))</f>
-        <v>46299</v>
+        <v>46303</v>
       </c>
       <c r="C22" s="6" t="str">
         <f>IF(Lists!$Q13="","",INDEX(Tasks[Task],Lists!$Q13)&amp;"")</f>
@@ -2313,7 +2313,7 @@
       <c r="A23" s="6"/>
       <c r="B23" s="33">
         <f>IF(Lists!$Q14="","",IF(MOD(INT(Lists!$P14),100000)=99999,"",MOD(INT(Lists!$P14),100000)))</f>
-        <v>46300</v>
+        <v>46304</v>
       </c>
       <c r="C23" s="6" t="str">
         <f>IF(Lists!$Q14="","",INDEX(Tasks[Task],Lists!$Q14)&amp;"")</f>
@@ -2364,7 +2364,7 @@
       <c r="A24" s="6"/>
       <c r="B24" s="33">
         <f>IF(Lists!$Q15="","",IF(MOD(INT(Lists!$P15),100000)=99999,"",MOD(INT(Lists!$P15),100000)))</f>
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="C24" s="6" t="str">
         <f>IF(Lists!$Q15="","",INDEX(Tasks[Task],Lists!$Q15)&amp;"")</f>
@@ -2421,7 +2421,7 @@
       <c r="A25" s="6"/>
       <c r="B25" s="33">
         <f>IF(Lists!$Q16="","",IF(MOD(INT(Lists!$P16),100000)=99999,"",MOD(INT(Lists!$P16),100000)))</f>
-        <v>46303</v>
+        <v>46307</v>
       </c>
       <c r="C25" s="6" t="str">
         <f>IF(Lists!$Q16="","",INDEX(Tasks[Task],Lists!$Q16)&amp;"")</f>
@@ -2486,7 +2486,7 @@
       <c r="A26" s="6"/>
       <c r="B26" s="33">
         <f>IF(Lists!$Q17="","",IF(MOD(INT(Lists!$P17),100000)=99999,"",MOD(INT(Lists!$P17),100000)))</f>
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="C26" s="6" t="str">
         <f>IF(Lists!$Q17="","",INDEX(Tasks[Task],Lists!$Q17)&amp;"")</f>
@@ -2551,7 +2551,7 @@
       <c r="A27" s="6"/>
       <c r="B27" s="33">
         <f>IF(Lists!$Q18="","",IF(MOD(INT(Lists!$P18),100000)=99999,"",MOD(INT(Lists!$P18),100000)))</f>
-        <v>46305</v>
+        <v>46309</v>
       </c>
       <c r="C27" s="6" t="str">
         <f>IF(Lists!$Q18="","",INDEX(Tasks[Task],Lists!$Q18)&amp;"")</f>
@@ -2791,7 +2791,7 @@
       <c r="A32" s="6"/>
       <c r="B32" s="33">
         <f ca="1">IF(Lists!$M4="","",INT(Lists!$L4))</f>
-        <v>46297</v>
+        <v>46301</v>
       </c>
       <c r="C32" s="6" t="str">
         <f ca="1">IF(Lists!$M4="","Nothing coming up",INDEX(Tasks[Task],Lists!$M4)&amp;"")</f>
@@ -2856,7 +2856,7 @@
       <c r="A33" s="6"/>
       <c r="B33" s="33">
         <f ca="1">IF(Lists!$M5="","",INT(Lists!$L5))</f>
-        <v>46298</v>
+        <v>46302</v>
       </c>
       <c r="C33" s="6" t="str">
         <f ca="1">IF(Lists!$M5="","",INDEX(Tasks[Task],Lists!$M5)&amp;"")</f>
@@ -2906,7 +2906,7 @@
       <c r="A34" s="6"/>
       <c r="B34" s="33">
         <f ca="1">IF(Lists!$M6="","",INT(Lists!$L6))</f>
-        <v>46299</v>
+        <v>46303</v>
       </c>
       <c r="C34" s="6" t="str">
         <f ca="1">IF(Lists!$M6="","",INDEX(Tasks[Task],Lists!$M6)&amp;"")</f>
@@ -2953,7 +2953,7 @@
       <c r="A35" s="6"/>
       <c r="B35" s="33">
         <f ca="1">IF(Lists!$M7="","",INT(Lists!$L7))</f>
-        <v>46300</v>
+        <v>46304</v>
       </c>
       <c r="C35" s="6" t="str">
         <f ca="1">IF(Lists!$M7="","",INDEX(Tasks[Task],Lists!$M7)&amp;"")</f>
@@ -3000,7 +3000,7 @@
       <c r="A36" s="6"/>
       <c r="B36" s="33">
         <f ca="1">IF(Lists!$M8="","",INT(Lists!$L8))</f>
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="C36" s="6" t="str">
         <f ca="1">IF(Lists!$M8="","",INDEX(Tasks[Task],Lists!$M8)&amp;"")</f>
@@ -3150,7 +3150,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E35422CB-ABC0-43BF-B8A7-FC3FE7104BBB}</x14:id>
+          <x14:id>{7DD9ADC7-A4BA-45BD-98C0-7C2567430AB9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -3164,7 +3164,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{25CF9E22-CE5E-445F-A44D-B79B8DAC43A1}</x14:id>
+          <x14:id>{DC98CC5B-160A-4530-85D9-83CF12364E09}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -3178,7 +3178,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{54681967-0840-4500-AD8C-E20FB4BA98A2}</x14:id>
+          <x14:id>{370AFC6A-8E62-419C-8606-93946B24281C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -3192,7 +3192,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C3C1AD25-AE66-42ED-BA09-341FB0F71CDD}</x14:id>
+          <x14:id>{D66F7962-E0DF-4356-B2EA-FDF4FA35A640}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -3242,13 +3242,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Owner" error="Pick a value from the list." sqref="C5" xr:uid="{4B2C24AC-35A5-4D3C-832A-AD0FB8D99A49}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Owner" error="Pick a value from the list." sqref="C5" xr:uid="{2652F965-A0B3-4ED3-98B7-D7A935E9CCD3}">
       <formula1>OwnerList</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Status" error="Pick a value from the list." sqref="E5" xr:uid="{8C4DEA33-04EC-4DEB-8BB7-BFEE728A8E1B}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Status" error="Pick a value from the list." sqref="E5" xr:uid="{F0C7AC77-2C2D-4B0B-88B1-EAE13F3A3DD7}">
       <formula1>StatusList</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Year" error="Pick a value from the list." sqref="H5" xr:uid="{86F91568-DA26-4F57-BE09-E76E98A91480}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Year" error="Pick a value from the list." sqref="H5" xr:uid="{C9CA92E9-D5EB-4A63-9DE9-FC9D72EB48BD}">
       <formula1>YearList</formula1>
     </dataValidation>
   </dataValidations>
@@ -3258,7 +3258,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E35422CB-ABC0-43BF-B8A7-FC3FE7104BBB}">
+          <x14:cfRule type="dataBar" id="{7DD9ADC7-A4BA-45BD-98C0-7C2567430AB9}">
             <x14:dataBar minLength="0" maxLength="100" gradient="0" negativeBarColorSameAsPositive="1" axisPosition="none">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -3271,7 +3271,7 @@
           <xm:sqref>I13:I27</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{25CF9E22-CE5E-445F-A44D-B79B8DAC43A1}">
+          <x14:cfRule type="dataBar" id="{DC98CC5B-160A-4530-85D9-83CF12364E09}">
             <x14:dataBar minLength="0" maxLength="100" gradient="0" negativeBarColorSameAsPositive="1" axisPosition="none">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -3284,7 +3284,7 @@
           <xm:sqref>I32:I36</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{54681967-0840-4500-AD8C-E20FB4BA98A2}">
+          <x14:cfRule type="dataBar" id="{370AFC6A-8E62-419C-8606-93946B24281C}">
             <x14:dataBar minLength="0" maxLength="100" gradient="0" negativeBarColorSameAsPositive="1" axisPosition="none">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -3297,7 +3297,7 @@
           <xm:sqref>Q13:Q20</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C3C1AD25-AE66-42ED-BA09-341FB0F71CDD}">
+          <x14:cfRule type="dataBar" id="{D66F7962-E0DF-4356-B2EA-FDF4FA35A640}">
             <x14:dataBar minLength="0" maxLength="100" gradient="0" negativeBarColorSameAsPositive="1" axisPosition="none">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -3316,7 +3316,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0E29D53-7DA7-496D-9574-91EDC903394C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE5E477B-3042-48D3-B78B-9A2FD1A0E76A}">
   <dimension ref="A1:K43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3386,10 +3386,10 @@
         <v>16</v>
       </c>
       <c r="G2" s="1">
-        <v>46237</v>
+        <v>46241</v>
       </c>
       <c r="H2" s="1">
-        <v>46262</v>
+        <v>46266</v>
       </c>
       <c r="I2" s="2">
         <v>1</v>
@@ -3422,10 +3422,10 @@
         <v>16</v>
       </c>
       <c r="G3" s="1">
-        <v>46252</v>
+        <v>46256</v>
       </c>
       <c r="H3" s="1">
-        <v>46269</v>
+        <v>46273</v>
       </c>
       <c r="I3" s="2">
         <v>1</v>
@@ -3455,10 +3455,10 @@
         <v>26</v>
       </c>
       <c r="G4" s="1">
-        <v>46257</v>
+        <v>46261</v>
       </c>
       <c r="H4" s="1">
-        <v>46276</v>
+        <v>46280</v>
       </c>
       <c r="I4" s="2">
         <v>1</v>
@@ -3491,10 +3491,10 @@
         <v>32</v>
       </c>
       <c r="G5" s="1">
-        <v>46267</v>
+        <v>46271</v>
       </c>
       <c r="H5" s="1">
-        <v>46283</v>
+        <v>46287</v>
       </c>
       <c r="I5" s="2">
         <v>1</v>
@@ -3524,10 +3524,10 @@
         <v>26</v>
       </c>
       <c r="G6" s="1">
-        <v>46272</v>
+        <v>46276</v>
       </c>
       <c r="H6" s="1">
-        <v>46288</v>
+        <v>46292</v>
       </c>
       <c r="I6" s="2">
         <v>1</v>
@@ -3557,10 +3557,10 @@
         <v>16</v>
       </c>
       <c r="G7" s="1">
-        <v>46267</v>
+        <v>46271</v>
       </c>
       <c r="H7" s="1">
-        <v>46285</v>
+        <v>46289</v>
       </c>
       <c r="I7" s="2">
         <v>0.7</v>
@@ -3593,10 +3593,10 @@
         <v>26</v>
       </c>
       <c r="G8" s="1">
-        <v>46269</v>
+        <v>46273</v>
       </c>
       <c r="H8" s="1">
-        <v>46289</v>
+        <v>46293</v>
       </c>
       <c r="I8" s="2">
         <v>0.6</v>
@@ -3626,10 +3626,10 @@
         <v>16</v>
       </c>
       <c r="G9" s="1">
-        <v>46277</v>
+        <v>46281</v>
       </c>
       <c r="H9" s="1">
-        <v>46291</v>
+        <v>46295</v>
       </c>
       <c r="I9" s="2">
         <v>0.4</v>
@@ -3662,10 +3662,10 @@
         <v>26</v>
       </c>
       <c r="G10" s="1">
-        <v>46276</v>
+        <v>46280</v>
       </c>
       <c r="H10" s="1">
-        <v>46293</v>
+        <v>46297</v>
       </c>
       <c r="I10" s="2">
         <v>0.8</v>
@@ -3695,10 +3695,10 @@
         <v>16</v>
       </c>
       <c r="G11" s="1">
-        <v>46287</v>
+        <v>46291</v>
       </c>
       <c r="H11" s="1">
-        <v>46295</v>
+        <v>46299</v>
       </c>
       <c r="I11" s="2">
         <v>0</v>
@@ -3728,10 +3728,10 @@
         <v>16</v>
       </c>
       <c r="G12" s="1">
-        <v>46288</v>
+        <v>46292</v>
       </c>
       <c r="H12" s="1">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="I12" s="2">
         <v>0.5</v>
@@ -3761,10 +3761,10 @@
         <v>26</v>
       </c>
       <c r="G13" s="1">
-        <v>46279</v>
+        <v>46283</v>
       </c>
       <c r="H13" s="1">
-        <v>46282</v>
+        <v>46286</v>
       </c>
       <c r="I13" s="2">
         <v>0.3</v>
@@ -3797,10 +3797,10 @@
         <v>26</v>
       </c>
       <c r="G14" s="1">
-        <v>46290</v>
+        <v>46294</v>
       </c>
       <c r="H14" s="1">
-        <v>46297</v>
+        <v>46301</v>
       </c>
       <c r="I14" s="2">
         <v>0.9</v>
@@ -3830,10 +3830,10 @@
         <v>32</v>
       </c>
       <c r="G15" s="1">
-        <v>46291</v>
+        <v>46295</v>
       </c>
       <c r="H15" s="1">
-        <v>46298</v>
+        <v>46302</v>
       </c>
       <c r="I15" s="2">
         <v>0.75</v>
@@ -3863,10 +3863,10 @@
         <v>16</v>
       </c>
       <c r="G16" s="1">
-        <v>46295</v>
+        <v>46299</v>
       </c>
       <c r="H16" s="1">
-        <v>46299</v>
+        <v>46303</v>
       </c>
       <c r="I16" s="2">
         <v>0</v>
@@ -3896,10 +3896,10 @@
         <v>26</v>
       </c>
       <c r="G17" s="1">
-        <v>46285</v>
+        <v>46289</v>
       </c>
       <c r="H17" s="1">
-        <v>46300</v>
+        <v>46304</v>
       </c>
       <c r="I17" s="2">
         <v>0.55000000000000004</v>
@@ -3929,10 +3929,10 @@
         <v>16</v>
       </c>
       <c r="G18" s="1">
-        <v>46289</v>
+        <v>46293</v>
       </c>
       <c r="H18" s="1">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="I18" s="2">
         <v>0.35</v>
@@ -3962,10 +3962,10 @@
         <v>16</v>
       </c>
       <c r="G19" s="1">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="H19" s="1">
-        <v>46303</v>
+        <v>46307</v>
       </c>
       <c r="I19" s="2">
         <v>0</v>
@@ -3995,10 +3995,10 @@
         <v>26</v>
       </c>
       <c r="G20" s="1">
-        <v>46287</v>
+        <v>46291</v>
       </c>
       <c r="H20" s="1">
-        <v>46299</v>
+        <v>46303</v>
       </c>
       <c r="I20" s="2">
         <v>1</v>
@@ -4031,10 +4031,10 @@
         <v>16</v>
       </c>
       <c r="G21" s="1">
-        <v>46283</v>
+        <v>46287</v>
       </c>
       <c r="H21" s="1">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="I21" s="2">
         <v>0.45</v>
@@ -4064,10 +4064,10 @@
         <v>26</v>
       </c>
       <c r="G22" s="1">
-        <v>46297</v>
+        <v>46301</v>
       </c>
       <c r="H22" s="1">
-        <v>46305</v>
+        <v>46309</v>
       </c>
       <c r="I22" s="2">
         <v>0</v>
@@ -4097,10 +4097,10 @@
         <v>32</v>
       </c>
       <c r="G23" s="1">
-        <v>46298</v>
+        <v>46302</v>
       </c>
       <c r="H23" s="1">
-        <v>46306</v>
+        <v>46310</v>
       </c>
       <c r="I23" s="2">
         <v>0</v>
@@ -4130,10 +4130,10 @@
         <v>16</v>
       </c>
       <c r="G24" s="1">
-        <v>46292</v>
+        <v>46296</v>
       </c>
       <c r="H24" s="1">
-        <v>46307</v>
+        <v>46311</v>
       </c>
       <c r="I24" s="2">
         <v>0.2</v>
@@ -4166,10 +4166,10 @@
         <v>16</v>
       </c>
       <c r="G25" s="1">
-        <v>46294</v>
+        <v>46298</v>
       </c>
       <c r="H25" s="1">
-        <v>46309</v>
+        <v>46313</v>
       </c>
       <c r="I25" s="2">
         <v>0.25</v>
@@ -4199,10 +4199,10 @@
         <v>26</v>
       </c>
       <c r="G26" s="1">
-        <v>46287</v>
+        <v>46291</v>
       </c>
       <c r="H26" s="1">
-        <v>46310</v>
+        <v>46314</v>
       </c>
       <c r="I26" s="2">
         <v>0.4</v>
@@ -4232,10 +4232,10 @@
         <v>16</v>
       </c>
       <c r="G27" s="1">
-        <v>46290</v>
+        <v>46294</v>
       </c>
       <c r="H27" s="1">
-        <v>46313</v>
+        <v>46317</v>
       </c>
       <c r="I27" s="2">
         <v>0.3</v>
@@ -4265,10 +4265,10 @@
         <v>26</v>
       </c>
       <c r="G28" s="1">
-        <v>46300</v>
+        <v>46304</v>
       </c>
       <c r="H28" s="1">
-        <v>46315</v>
+        <v>46319</v>
       </c>
       <c r="I28" s="2">
         <v>0</v>
@@ -4298,10 +4298,10 @@
         <v>26</v>
       </c>
       <c r="G29" s="1">
-        <v>46293</v>
+        <v>46297</v>
       </c>
       <c r="H29" s="1">
-        <v>46318</v>
+        <v>46322</v>
       </c>
       <c r="I29" s="2">
         <v>0.15</v>
@@ -4331,10 +4331,10 @@
         <v>16</v>
       </c>
       <c r="G30" s="1">
-        <v>46317</v>
+        <v>46321</v>
       </c>
       <c r="H30" s="1">
-        <v>46324</v>
+        <v>46328</v>
       </c>
       <c r="I30" s="2">
         <v>0</v>
@@ -4364,10 +4364,10 @@
         <v>26</v>
       </c>
       <c r="G31" s="1">
-        <v>46295</v>
+        <v>46299</v>
       </c>
       <c r="H31" s="1">
-        <v>46327</v>
+        <v>46331</v>
       </c>
       <c r="I31" s="2">
         <v>0.2</v>
@@ -4397,10 +4397,10 @@
         <v>26</v>
       </c>
       <c r="G32" s="1">
-        <v>46282</v>
+        <v>46286</v>
       </c>
       <c r="H32" s="1">
-        <v>46332</v>
+        <v>46336</v>
       </c>
       <c r="I32" s="2">
         <v>0.1</v>
@@ -4433,10 +4433,10 @@
         <v>16</v>
       </c>
       <c r="G33" s="1">
-        <v>46307</v>
+        <v>46311</v>
       </c>
       <c r="H33" s="1">
-        <v>46339</v>
+        <v>46343</v>
       </c>
       <c r="I33" s="2">
         <v>0</v>
@@ -4466,10 +4466,10 @@
         <v>32</v>
       </c>
       <c r="G34" s="1">
-        <v>46285</v>
+        <v>46289</v>
       </c>
       <c r="H34" s="1">
-        <v>46311</v>
+        <v>46315</v>
       </c>
       <c r="I34" s="2">
         <v>1</v>
@@ -4499,10 +4499,10 @@
         <v>26</v>
       </c>
       <c r="G35" s="1">
-        <v>46291</v>
+        <v>46295</v>
       </c>
       <c r="H35" s="1">
-        <v>46345</v>
+        <v>46349</v>
       </c>
       <c r="I35" s="2">
         <v>0.1</v>
@@ -4532,10 +4532,10 @@
         <v>32</v>
       </c>
       <c r="G36" s="1">
-        <v>46311</v>
+        <v>46315</v>
       </c>
       <c r="H36" s="1">
-        <v>46353</v>
+        <v>46357</v>
       </c>
       <c r="I36" s="2">
         <v>0</v>
@@ -4565,10 +4565,10 @@
         <v>26</v>
       </c>
       <c r="G37" s="1">
-        <v>46262</v>
+        <v>46266</v>
       </c>
       <c r="H37" s="1">
-        <v>46279</v>
+        <v>46283</v>
       </c>
       <c r="I37" s="2">
         <v>1</v>
@@ -4598,10 +4598,10 @@
         <v>16</v>
       </c>
       <c r="G38" s="1">
-        <v>46277</v>
+        <v>46281</v>
       </c>
       <c r="H38" s="1">
-        <v>46292</v>
+        <v>46296</v>
       </c>
       <c r="I38" s="2">
         <v>1</v>
@@ -4631,10 +4631,10 @@
         <v>16</v>
       </c>
       <c r="G39" s="1">
-        <v>46357</v>
+        <v>46361</v>
       </c>
       <c r="H39" s="1">
-        <v>46392</v>
+        <v>46396</v>
       </c>
       <c r="I39" s="2">
         <v>0</v>
@@ -4664,10 +4664,10 @@
         <v>32</v>
       </c>
       <c r="G40" s="1">
-        <v>46367</v>
+        <v>46371</v>
       </c>
       <c r="H40" s="1">
-        <v>46397</v>
+        <v>46401</v>
       </c>
       <c r="I40" s="2">
         <v>0</v>
@@ -4697,10 +4697,10 @@
         <v>26</v>
       </c>
       <c r="G41" s="1">
-        <v>46362</v>
+        <v>46366</v>
       </c>
       <c r="H41" s="1">
-        <v>46402</v>
+        <v>46406</v>
       </c>
       <c r="I41" s="2">
         <v>0</v>
@@ -4730,10 +4730,10 @@
         <v>26</v>
       </c>
       <c r="G42" s="1">
-        <v>46377</v>
+        <v>46381</v>
       </c>
       <c r="H42" s="1">
-        <v>46415</v>
+        <v>46419</v>
       </c>
       <c r="I42" s="2">
         <v>0</v>
@@ -4763,10 +4763,10 @@
         <v>32</v>
       </c>
       <c r="G43" s="1">
-        <v>46327</v>
+        <v>46331</v>
       </c>
       <c r="H43" s="1">
-        <v>46422</v>
+        <v>46426</v>
       </c>
       <c r="I43" s="2">
         <v>0.05</v>
@@ -4789,17 +4789,17 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Status" error="Pick one of: Not started, In progress, Blocked, Done" sqref="E2:E43" xr:uid="{489FB4ED-78EE-4EAF-BA4F-29FF421A5E55}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Status" error="Pick one of: Not started, In progress, Blocked, Done" sqref="E2:E43" xr:uid="{7DD60231-D010-4DEC-BC9F-E510163CA591}">
       <formula1>"Not started,In progress,Blocked,Done"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Priority" error="Pick one of: High, Medium, Low" sqref="F2:F43" xr:uid="{DC4C2EF8-47B8-4000-B5A7-7781B7C1AFB7}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Priority" error="Pick one of: High, Medium, Low" sqref="F2:F43" xr:uid="{063D0543-70EA-4E80-BC6B-88278773C6D1}">
       <formula1>"High,Medium,Low"</formula1>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="% Complete" error="Type a percentage from 0% to 100%." sqref="I2:I43" xr:uid="{17A0DE7D-172C-476A-ABB0-6A858CB2A8E6}">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="% Complete" error="Type a percentage from 0% to 100%." sqref="I2:I43" xr:uid="{65C1A00B-3971-4BBB-98F9-F5F8BA6AFB4E}">
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Year" prompt="Calculated: fills itself in from Due. No need to type here." sqref="J2:J43" xr:uid="{49644272-0EEF-432C-8DF6-DFD975428AA1}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Year" prompt="Calculated: fills itself in from Due. No need to type here." sqref="J2:J43" xr:uid="{AFE86B2E-D0E4-450A-B66E-64459ADB78E2}"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -4809,7 +4809,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98B8A97E-0897-4869-9F80-D3A8E4EEEED7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1F64F9D-DA22-4008-B9C0-1CC36293FDCE}">
   <dimension ref="B1:C30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4973,7 +4973,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5635006D-7825-4AB4-BCB0-0E46EA8A39F4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D1CAF32-C6C9-4BF7-B6E5-B4DE9DE86E02}">
   <sheetPr>
     <tabColor rgb="FF5B6B7F"/>
   </sheetPr>
@@ -5062,7 +5062,7 @@
       </c>
       <c r="H4" s="14">
         <f ca="1">IFERROR(_xlfn.AGGREGATE(15,6,SortKey/CondFocus,$G4),"")</f>
-        <v>46297.00013</v>
+        <v>46301.00013</v>
       </c>
       <c r="I4">
         <f t="shared" ref="I4:I11" ca="1" si="0">IF(H4="","",ROUND(MOD(H4,1)*100000,0))</f>
@@ -5073,7 +5073,7 @@
       </c>
       <c r="L4" s="14">
         <f ca="1">IFERROR(_xlfn.AGGREGATE(15,6,SortKey/CondUpcoming,$K4),"")</f>
-        <v>46297.00013</v>
+        <v>46301.00013</v>
       </c>
       <c r="M4">
         <f t="shared" ref="M4:M8" ca="1" si="1">IF(L4="","",ROUND(MOD(L4,1)*100000,0))</f>
@@ -5084,7 +5084,7 @@
       </c>
       <c r="P4" s="14">
         <f>IFERROR(_xlfn.AGGREGATE(15,6,SortKeyView/InScope,$O4),"")</f>
-        <v>46282.000119999997</v>
+        <v>46286.000119999997</v>
       </c>
       <c r="Q4">
         <f t="shared" ref="Q4:Q18" si="2">IF(P4="","",ROUND(MOD(P4,1)*100000,0))</f>
@@ -5108,7 +5108,7 @@
       </c>
       <c r="H5" s="14">
         <f ca="1">IFERROR(_xlfn.AGGREGATE(15,6,SortKey/CondFocus,$G5),"")</f>
-        <v>46298.000139999996</v>
+        <v>46302.000139999996</v>
       </c>
       <c r="I5">
         <f t="shared" ca="1" si="0"/>
@@ -5119,7 +5119,7 @@
       </c>
       <c r="L5" s="14">
         <f ca="1">IFERROR(_xlfn.AGGREGATE(15,6,SortKey/CondUpcoming,$K5),"")</f>
-        <v>46298.000139999996</v>
+        <v>46302.000139999996</v>
       </c>
       <c r="M5">
         <f t="shared" ca="1" si="1"/>
@@ -5130,7 +5130,7 @@
       </c>
       <c r="P5" s="14">
         <f>IFERROR(_xlfn.AGGREGATE(15,6,SortKeyView/InScope,$O5),"")</f>
-        <v>46285.000059999998</v>
+        <v>46289.000059999998</v>
       </c>
       <c r="Q5">
         <f t="shared" si="2"/>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="H6" s="14">
         <f ca="1">IFERROR(_xlfn.AGGREGATE(15,6,SortKey/CondFocus,$G6),"")</f>
-        <v>46299.00015</v>
+        <v>46303.00015</v>
       </c>
       <c r="I6">
         <f t="shared" ca="1" si="0"/>
@@ -5165,7 +5165,7 @@
       </c>
       <c r="L6" s="14">
         <f ca="1">IFERROR(_xlfn.AGGREGATE(15,6,SortKey/CondUpcoming,$K6),"")</f>
-        <v>46299.00015</v>
+        <v>46303.00015</v>
       </c>
       <c r="M6">
         <f t="shared" ca="1" si="1"/>
@@ -5176,7 +5176,7 @@
       </c>
       <c r="P6" s="14">
         <f>IFERROR(_xlfn.AGGREGATE(15,6,SortKeyView/InScope,$O6),"")</f>
-        <v>46289.000070000002</v>
+        <v>46293.000070000002</v>
       </c>
       <c r="Q6">
         <f t="shared" si="2"/>
@@ -5200,7 +5200,7 @@
       </c>
       <c r="H7" s="14">
         <f ca="1">IFERROR(_xlfn.AGGREGATE(15,6,SortKey/CondFocus,$G7),"")</f>
-        <v>46300.000160000003</v>
+        <v>46304.000160000003</v>
       </c>
       <c r="I7">
         <f t="shared" ca="1" si="0"/>
@@ -5211,7 +5211,7 @@
       </c>
       <c r="L7" s="14">
         <f ca="1">IFERROR(_xlfn.AGGREGATE(15,6,SortKey/CondUpcoming,$K7),"")</f>
-        <v>46300.000160000003</v>
+        <v>46304.000160000003</v>
       </c>
       <c r="M7">
         <f t="shared" ca="1" si="1"/>
@@ -5222,7 +5222,7 @@
       </c>
       <c r="P7" s="14">
         <f>IFERROR(_xlfn.AGGREGATE(15,6,SortKeyView/InScope,$O7),"")</f>
-        <v>46291.000079999998</v>
+        <v>46295.000079999998</v>
       </c>
       <c r="Q7">
         <f t="shared" si="2"/>
@@ -5246,7 +5246,7 @@
       </c>
       <c r="H8" s="14">
         <f ca="1">IFERROR(_xlfn.AGGREGATE(15,6,SortKey/CondFocus,$G8),"")</f>
-        <v>46302.000169999999</v>
+        <v>46306.000169999999</v>
       </c>
       <c r="I8">
         <f t="shared" ca="1" si="0"/>
@@ -5257,7 +5257,7 @@
       </c>
       <c r="L8" s="14">
         <f ca="1">IFERROR(_xlfn.AGGREGATE(15,6,SortKey/CondUpcoming,$K8),"")</f>
-        <v>46302.000169999999</v>
+        <v>46306.000169999999</v>
       </c>
       <c r="M8">
         <f t="shared" ca="1" si="1"/>
@@ -5268,7 +5268,7 @@
       </c>
       <c r="P8" s="14">
         <f>IFERROR(_xlfn.AGGREGATE(15,6,SortKeyView/InScope,$O8),"")</f>
-        <v>46293.000090000001</v>
+        <v>46297.000090000001</v>
       </c>
       <c r="Q8">
         <f t="shared" si="2"/>
@@ -5289,7 +5289,7 @@
       </c>
       <c r="H9" s="14">
         <f ca="1">IFERROR(_xlfn.AGGREGATE(15,6,SortKey/CondFocus,$G9),"")</f>
-        <v>46303.000180000003</v>
+        <v>46307.000180000003</v>
       </c>
       <c r="I9">
         <f t="shared" ca="1" si="0"/>
@@ -5300,7 +5300,7 @@
       </c>
       <c r="P9" s="14">
         <f>IFERROR(_xlfn.AGGREGATE(15,6,SortKeyView/InScope,$O9),"")</f>
-        <v>46295.000099999997</v>
+        <v>46299.000099999997</v>
       </c>
       <c r="Q9">
         <f t="shared" si="2"/>
@@ -5332,7 +5332,7 @@
       </c>
       <c r="P10" s="14">
         <f>IFERROR(_xlfn.AGGREGATE(15,6,SortKeyView/InScope,$O10),"")</f>
-        <v>46296.000110000001</v>
+        <v>46300.000110000001</v>
       </c>
       <c r="Q10">
         <f t="shared" si="2"/>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="P11" s="14">
         <f>IFERROR(_xlfn.AGGREGATE(15,6,SortKeyView/InScope,$O11),"")</f>
-        <v>46297.00013</v>
+        <v>46301.00013</v>
       </c>
       <c r="Q11">
         <f t="shared" si="2"/>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="P12" s="14">
         <f>IFERROR(_xlfn.AGGREGATE(15,6,SortKeyView/InScope,$O12),"")</f>
-        <v>46298.000139999996</v>
+        <v>46302.000139999996</v>
       </c>
       <c r="Q12">
         <f t="shared" si="2"/>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="P13" s="14">
         <f>IFERROR(_xlfn.AGGREGATE(15,6,SortKeyView/InScope,$O13),"")</f>
-        <v>46299.00015</v>
+        <v>46303.00015</v>
       </c>
       <c r="Q13">
         <f t="shared" si="2"/>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="P14" s="14">
         <f>IFERROR(_xlfn.AGGREGATE(15,6,SortKeyView/InScope,$O14),"")</f>
-        <v>46300.000160000003</v>
+        <v>46304.000160000003</v>
       </c>
       <c r="Q14">
         <f t="shared" si="2"/>
@@ -5444,7 +5444,7 @@
       </c>
       <c r="P15" s="14">
         <f>IFERROR(_xlfn.AGGREGATE(15,6,SortKeyView/InScope,$O15),"")</f>
-        <v>46302.000169999999</v>
+        <v>46306.000169999999</v>
       </c>
       <c r="Q15">
         <f t="shared" si="2"/>
@@ -5461,7 +5461,7 @@
       </c>
       <c r="P16" s="14">
         <f>IFERROR(_xlfn.AGGREGATE(15,6,SortKeyView/InScope,$O16),"")</f>
-        <v>46303.000180000003</v>
+        <v>46307.000180000003</v>
       </c>
       <c r="Q16">
         <f t="shared" si="2"/>
@@ -5478,7 +5478,7 @@
       </c>
       <c r="P17" s="14">
         <f>IFERROR(_xlfn.AGGREGATE(15,6,SortKeyView/InScope,$O17),"")</f>
-        <v>46304.000200000002</v>
+        <v>46308.000200000002</v>
       </c>
       <c r="Q17">
         <f t="shared" si="2"/>
@@ -5495,7 +5495,7 @@
       </c>
       <c r="P18" s="14">
         <f>IFERROR(_xlfn.AGGREGATE(15,6,SortKeyView/InScope,$O18),"")</f>
-        <v>46305.000209999998</v>
+        <v>46309.000209999998</v>
       </c>
       <c r="Q18">
         <f t="shared" si="2"/>

</xml_diff>